<commit_message>
Afegida Variació P i G en cartera any.
--HG--
branch : Simplifico PiG
</commit_message>
<xml_diff>
--- a/Docs/CanvisEnCalculPiGCompra.xlsx
+++ b/Docs/CanvisEnCalculPiGCompra.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193EA251-8A9E-4D46-A8EB-DD2EEDA66533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{052458C3-D00C-45F8-8549-662EFA69C845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{F98390CD-C643-446D-B540-89851331605B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="19-NB Capital Plus FI" sheetId="3" r:id="rId2"/>
-    <sheet name="Aktien" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="4" r:id="rId2"/>
+    <sheet name="19-NB Capital Plus FI" sheetId="3" r:id="rId3"/>
+    <sheet name="Aktien" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="41">
   <si>
     <t>Orig</t>
   </si>
@@ -137,19 +138,41 @@
   </si>
   <si>
     <t>PiG</t>
+  </si>
+  <si>
+    <t>Deutschland</t>
+  </si>
+  <si>
+    <t>DWS Aktien Strategie Deutschland</t>
+  </si>
+  <si>
+    <t>NB Capital Plus FI</t>
+  </si>
+  <si>
+    <t>CS Corto Plazo B FI</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>PU Inici</t>
+  </si>
+  <si>
+    <t>PU Act</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000"/>
-    <numFmt numFmtId="170" formatCode="#,##0.000\ &quot;€&quot;;[Red]\-#,##0.000\ &quot;€&quot;"/>
+    <numFmt numFmtId="166" formatCode="#,##0.000\ &quot;€&quot;;[Red]\-#,##0.000\ &quot;€&quot;"/>
+    <numFmt numFmtId="172" formatCode="#,##0.0000\ &quot;€&quot;;[Red]\-#,##0.0000\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +182,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -183,10 +213,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -221,10 +252,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -536,7 +582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB91E7F3-6CE6-4994-A1EF-34CFE36D11EB}">
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.08984375" customWidth="1"/>
@@ -550,18 +596,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="15"/>
-      <c r="E1" s="15" t="s">
+      <c r="C1" s="17"/>
+      <c r="E1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="15"/>
-      <c r="H1" s="15" t="s">
+      <c r="F1" s="17"/>
+      <c r="H1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="15"/>
+      <c r="I1" s="17"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -789,7 +835,7 @@
         <v>-696.75</v>
       </c>
       <c r="I12" s="1">
-        <f>F12-C3</f>
+        <f t="shared" ref="I12:I17" si="4">F12-C3</f>
         <v>-3.0000000000029559E-2</v>
       </c>
     </row>
@@ -810,7 +856,7 @@
         <v>702.23</v>
       </c>
       <c r="I13" s="1">
-        <f>F13-C4</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -831,7 +877,7 @@
         <v>-9.9999999999909051E-3</v>
       </c>
       <c r="I14" s="1">
-        <f>F14-C5</f>
+        <f t="shared" si="4"/>
         <v>-0.18999999999999773</v>
       </c>
     </row>
@@ -852,7 +898,7 @@
         <v>-382.97999999999956</v>
       </c>
       <c r="I15" s="1">
-        <f>F15-C6</f>
+        <f t="shared" si="4"/>
         <v>-0.13999999999998636</v>
       </c>
     </row>
@@ -873,7 +919,7 @@
         <v>1.0300000000024738</v>
       </c>
       <c r="I16" s="1">
-        <f>F16-C7</f>
+        <f t="shared" si="4"/>
         <v>2.9999999998835847E-2</v>
       </c>
     </row>
@@ -894,7 +940,7 @@
         <v>-2.0299999999997453</v>
       </c>
       <c r="I17" s="1">
-        <f>F17-C8</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -921,11 +967,11 @@
         <v>-325.98</v>
       </c>
       <c r="H20" s="1">
-        <f>E20-B3</f>
+        <f t="shared" ref="H20:I25" si="5">E20-B3</f>
         <v>-696.75</v>
       </c>
       <c r="I20" s="1">
-        <f>F20-C3</f>
+        <f t="shared" si="5"/>
         <v>-3.0000000000029559E-2</v>
       </c>
     </row>
@@ -940,11 +986,11 @@
         <v>-364.32</v>
       </c>
       <c r="H21" s="1">
-        <f>E21-B4</f>
+        <f t="shared" si="5"/>
         <v>702.23</v>
       </c>
       <c r="I21" s="1">
-        <f>F21-C4</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -959,11 +1005,11 @@
         <v>308.2</v>
       </c>
       <c r="H22" s="1">
-        <f>E22-B5</f>
+        <f t="shared" si="5"/>
         <v>-9.9999999999909051E-3</v>
       </c>
       <c r="I22" s="1">
-        <f>F22-C5</f>
+        <f t="shared" si="5"/>
         <v>-0.18999999999999773</v>
       </c>
     </row>
@@ -978,11 +1024,11 @@
         <v>-151.63</v>
       </c>
       <c r="H23" s="1">
-        <f>E23-B6</f>
+        <f t="shared" si="5"/>
         <v>-382.97999999999956</v>
       </c>
       <c r="I23" s="1">
-        <f>F23-C6</f>
+        <f t="shared" si="5"/>
         <v>-0.13999999999998636</v>
       </c>
     </row>
@@ -997,11 +1043,11 @@
         <v>17961.03</v>
       </c>
       <c r="H24" s="1">
-        <f>E24-B7</f>
+        <f t="shared" si="5"/>
         <v>1.0300000000024738</v>
       </c>
       <c r="I24" s="1">
-        <f>F24-C7</f>
+        <f t="shared" si="5"/>
         <v>2.9999999998835847E-2</v>
       </c>
     </row>
@@ -1016,11 +1062,11 @@
         <v>3363.25</v>
       </c>
       <c r="H25" s="1">
-        <f>E25-B8</f>
+        <f t="shared" si="5"/>
         <v>-2.0299999999997453</v>
       </c>
       <c r="I25" s="1">
-        <f>F25-C8</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1034,9 +1080,20 @@
         <v>-378.50999999999681</v>
       </c>
     </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="F29">
+        <v>435.09140000000002</v>
+      </c>
+    </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B30" s="13">
         <v>1846.86</v>
+      </c>
+      <c r="E30" s="23">
+        <v>44473</v>
+      </c>
+      <c r="F30" s="24">
+        <v>435.1019</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
@@ -1053,10 +1110,15 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C33">
         <f>+B32-C32</f>
         <v>-7.3127500000000509</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B35" s="18">
+        <v>1898.4177999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1071,6 +1133,306 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF98832-DB2E-4AF9-8761-89A3EDDF212E}">
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="44.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="1.26953125" customWidth="1"/>
+    <col min="7" max="7" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="C1" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="1">
+        <v>-249.38</v>
+      </c>
+      <c r="C2" s="18">
+        <v>280.14</v>
+      </c>
+      <c r="D2" s="18">
+        <v>230.24</v>
+      </c>
+      <c r="E2">
+        <v>4.9976000000000003</v>
+      </c>
+      <c r="G2" s="1">
+        <f>(D2-C2)*E2</f>
+        <v>-249.3802399999999</v>
+      </c>
+      <c r="H2" s="21">
+        <f>D2/C2-1</f>
+        <v>-0.17812522310273426</v>
+      </c>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="1">
+        <v>-2754.25</v>
+      </c>
+      <c r="C3" s="18">
+        <v>568.23</v>
+      </c>
+      <c r="D3" s="18">
+        <v>458.06</v>
+      </c>
+      <c r="E3">
+        <v>25</v>
+      </c>
+      <c r="G3" s="1">
+        <f t="shared" ref="G3:G7" si="0">(D3-C3)*E3</f>
+        <v>-2754.2500000000005</v>
+      </c>
+      <c r="H3" s="21">
+        <f t="shared" ref="H3:H8" si="1">D3/C3-1</f>
+        <v>-0.19388275874205874</v>
+      </c>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="1">
+        <v>-318.2</v>
+      </c>
+      <c r="C4" s="18">
+        <v>1898.4177999999999</v>
+      </c>
+      <c r="D4" s="18">
+        <v>1846.86</v>
+      </c>
+      <c r="E4">
+        <v>6.1711</v>
+      </c>
+      <c r="G4" s="1">
+        <f t="shared" si="0"/>
+        <v>-318.16833958000029</v>
+      </c>
+      <c r="H4" s="21">
+        <f t="shared" si="1"/>
+        <v>-2.7158299927444896E-2</v>
+      </c>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1">
+        <v>-6529.09</v>
+      </c>
+      <c r="C5" s="18">
+        <v>37.380000000000003</v>
+      </c>
+      <c r="D5" s="18">
+        <v>31.96</v>
+      </c>
+      <c r="E5" s="13">
+        <v>1204.6300000000001</v>
+      </c>
+      <c r="G5" s="1">
+        <f t="shared" si="0"/>
+        <v>-6529.0946000000031</v>
+      </c>
+      <c r="H5" s="21">
+        <f t="shared" si="1"/>
+        <v>-0.14499732477260574</v>
+      </c>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1">
+        <v>-107.63</v>
+      </c>
+      <c r="C6" s="18">
+        <v>434.483</v>
+      </c>
+      <c r="D6" s="18">
+        <v>433.46</v>
+      </c>
+      <c r="E6">
+        <v>105.53</v>
+      </c>
+      <c r="G6" s="1">
+        <f t="shared" si="0"/>
+        <v>-107.9571900000026</v>
+      </c>
+      <c r="H6" s="21">
+        <f t="shared" si="1"/>
+        <v>-2.3545225014558469E-3</v>
+      </c>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="1">
+        <v>-352.99</v>
+      </c>
+      <c r="C7" s="18">
+        <v>13.024699999999999</v>
+      </c>
+      <c r="D7" s="18">
+        <v>12.563499999999999</v>
+      </c>
+      <c r="E7">
+        <v>765.3691</v>
+      </c>
+      <c r="G7" s="1">
+        <f t="shared" si="0"/>
+        <v>-352.98822891999987</v>
+      </c>
+      <c r="H7" s="21">
+        <f t="shared" si="1"/>
+        <v>-3.5409644751894453E-2</v>
+      </c>
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="4">
+        <v>-10311.540000000001</v>
+      </c>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="2"/>
+      <c r="G8" s="4">
+        <f>SUM(G2:G7)</f>
+        <v>-10311.838598500006</v>
+      </c>
+      <c r="H8" s="20"/>
+      <c r="I8" s="1"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="1">
+        <v>-249.38</v>
+      </c>
+      <c r="C10" s="22">
+        <v>-0.17810000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="1">
+        <v>-2754.25</v>
+      </c>
+      <c r="C11" s="22">
+        <v>-0.19389999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="1">
+        <v>-318.2</v>
+      </c>
+      <c r="C12" s="22">
+        <v>-2.7199999999999998E-2</v>
+      </c>
+      <c r="G12" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="1">
+        <v>-6529.09</v>
+      </c>
+      <c r="C13" s="22">
+        <v>-0.14499999999999999</v>
+      </c>
+      <c r="G13" s="1">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="1">
+        <v>-107.63</v>
+      </c>
+      <c r="C14" s="22">
+        <v>-2.3E-3</v>
+      </c>
+      <c r="G14">
+        <f>SUM(G12:G13)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" s="1">
+        <v>-352.99</v>
+      </c>
+      <c r="C15" s="22">
+        <v>-3.5400000000000001E-2</v>
+      </c>
+      <c r="G15" s="1">
+        <f>(D3-C3)*G14</f>
+        <v>-6059.3500000000013</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="1">
+        <v>-10311.540000000001</v>
+      </c>
+      <c r="G16" s="1">
+        <v>-3111.41</v>
+      </c>
+    </row>
+    <row r="17" spans="7:7" x14ac:dyDescent="0.35">
+      <c r="G17" s="1">
+        <f>+G15+G16</f>
+        <v>-9170.760000000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F14FBE7-6DCA-4EF8-BD6D-488C6DB64216}">
   <dimension ref="A1:N12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1169,7 +1531,7 @@
         <v>886.59</v>
       </c>
       <c r="H3" s="10">
-        <f t="shared" ref="H3:H5" si="0">E3*F$5</f>
+        <f t="shared" ref="H3:H4" si="0">E3*F$5</f>
         <v>863.96110799999997</v>
       </c>
       <c r="I3" s="8">
@@ -1405,7 +1767,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D7359EB-DCDD-42EB-8735-4CF6CA83B044}">
   <dimension ref="A1:R11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>